<commit_message>
Execute Login test cases and refine wording
</commit_message>
<xml_diff>
--- a/Test-Cases/Test-Cases-Login.xlsx
+++ b/Test-Cases/Test-Cases-Login.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0. Documentos\Github\qa-saucedemo-testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42172F7E-E3C0-4FFF-AB4F-65F6AF35AC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{666A3B4A-31D8-42E7-8C5B-B1A27D460A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
   <si>
     <t>ID</t>
   </si>
@@ -63,16 +63,6 @@
     <t>High</t>
   </si>
   <si>
-    <t>Given the user is on the SauceDemo login page
-When they enter "standard_user" in the Username field
-And they enter "secret_sauce" in the Password field
-And they click the "Login" button
-Then the system redirects them to the inventory page (/inventory.html)</t>
-  </si>
-  <si>
-    <t>Pending</t>
-  </si>
-  <si>
     <t>TC-002</t>
   </si>
   <si>
@@ -82,13 +72,6 @@
     <t>Functional / Negative</t>
   </si>
   <si>
-    <t>Given the user is on the login page
-When they enter "standard_user" in the Username field
-And they leave the Password field empty
-And they click the "Login" button
-Then the system displays the message "Epic sadface: Password is required"</t>
-  </si>
-  <si>
     <t>TC-003</t>
   </si>
   <si>
@@ -98,13 +81,6 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>Given the user is on the login page
-When they leave the Username field empty
-And they enter "secret_sauce" in the Password field
-And they click the "Login" button
-Then the system displays the message "Epic sadface: Password is required"</t>
-  </si>
-  <si>
     <t>TC-004</t>
   </si>
   <si>
@@ -114,36 +90,16 @@
     <t>Edge case</t>
   </si>
   <si>
-    <t>Given the user is on the login page
-When they leave both the Username and Password fields empty
-And they click the "Login" button
-Then the system displays the message "Epic sadface: Username is required"</t>
-  </si>
-  <si>
     <t>TC-005</t>
   </si>
   <si>
     <t>Login with locked out user</t>
   </si>
   <si>
-    <t>Given the user is on the login page
-When they enter "locked_out_user" in the Username field
-And they enter "secret_sauce" in the Password field
-And they click the "Login" button
-Then the system displays the message "Epic sadface: Sorry, this user has been locked out."</t>
-  </si>
-  <si>
     <t>TC-006</t>
   </si>
   <si>
     <t>Login with uppercase username (case sensitivity)</t>
-  </si>
-  <si>
-    <t>Given the user is on the login page
-When they enter "Standard_user" in the Username field (with an initial capital letter)
-And they enter "secret_sauce" in the Password field
-And they click the "Login" button
-Then the system displays the message "Epic sadface: Username and password do not match any user in this service"</t>
   </si>
   <si>
     <t>TC-007</t>
@@ -166,6 +122,62 @@
   </si>
   <si>
     <t>The login was rejected and the generic message was displayed.</t>
+  </si>
+  <si>
+    <t>The user is redirected to the inventory page (/inventory.html).</t>
+  </si>
+  <si>
+    <t>Given the user is on the SauceDemo login page
+When they enter "standard_user" in the Username field
+And they enter "secret_sauce" in the Password field
+And they click the "Login" button
+Then the system should redirect them to the inventory page (/inventory.html)</t>
+  </si>
+  <si>
+    <t>Given the user is on the login page
+When they enter "standard_user" in the Username field
+And they leave the Password field empty
+And they click the "Login" button
+Then the system should display the message "Epic sadface: Password is required"</t>
+  </si>
+  <si>
+    <t>Given the user is on the login page
+When they leave the Username field empty
+And they enter "secret_sauce" in the Password field
+And they click the "Login" button
+Then the system should display the message "Epic sadface: Username is required"</t>
+  </si>
+  <si>
+    <t>Given the user is on the login page
+When they leave both the Username and Password fields empty
+And they click the "Login" button
+Then the system should display the message "Epic sadface: Username is required"</t>
+  </si>
+  <si>
+    <t>Given the user is on the login page
+When they enter "locked_out_user" in the Username field
+And they enter "secret_sauce" in the Password field
+And they click the "Login" button
+Then the system should display the message "Epic sadface: Sorry, this user has been locked out."</t>
+  </si>
+  <si>
+    <t>Given the user is on the login page
+When they enter "Standard_user" in the Username field (with an initial capital letter)
+And they enter "secret_sauce" in the Password field
+And they click the "Login" button
+Then the system should display the message "Epic sadface: Username and password do not match any user in this service"</t>
+  </si>
+  <si>
+    <t>The login was rejected and the system displayed "Epic sadface: Password is required".</t>
+  </si>
+  <si>
+    <t>The login was rejected and the system displayed "Epic sadface: Username is required".</t>
+  </si>
+  <si>
+    <t>The login was rejected and the system displayed "Epic sadface: Sorry, this user has been locked out."</t>
+  </si>
+  <si>
+    <t>The login was rejected and the system displayed "Epic sadface: Username and password do not match any user in this service".</t>
   </si>
 </sst>
 </file>
@@ -282,7 +294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -311,7 +323,13 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -585,7 +603,8 @@
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="78" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
-    <col min="7" max="8" width="14" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="14" style="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -610,7 +629,7 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -628,147 +647,173 @@
         <v>11</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="G2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="H2" s="10">
+        <v>46304</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="3"/>
+        <v>33</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>38</v>
+      </c>
       <c r="G3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="H3" s="10">
+        <v>46304</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>39</v>
+      </c>
       <c r="G4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="H4" s="10">
+        <v>46304</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="10">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="84.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>27</v>
-      </c>
       <c r="C6" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" s="3"/>
+        <v>36</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="G6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="H6" s="10">
+        <v>46304</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="82.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="10">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="F8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" s="10" customFormat="1" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>37</v>
-      </c>
       <c r="G8" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="H8" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="H8" s="10">
+        <v>46304</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>